<commit_message>
Daily NSE delivery update
</commit_message>
<xml_diff>
--- a/data/nse/delivery/daily_output/delivery_breakout_20260520.xlsx
+++ b/data/nse/delivery/daily_output/delivery_breakout_20260520.xlsx
@@ -425,19 +425,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,36 +455,6 @@
           <t>DELIVERY_RATIO</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>DELIV_PER</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>TTL_TRD_QNTY</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>AVG_30_VOLUME</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>VOLUME_RATIO</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>CLOSE_PRICE</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>PRICE_CHANGE</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -506,89 +470,230 @@
       <c r="D2" t="n">
         <v>11.5</v>
       </c>
-      <c r="E2" t="n">
-        <v>67.95</v>
-      </c>
-      <c r="F2" t="n">
-        <v>633794</v>
-      </c>
-      <c r="G2" t="n">
-        <v>64450.62068965517</v>
-      </c>
-      <c r="H2" t="n">
-        <v>9.83</v>
-      </c>
-      <c r="I2" t="n">
-        <v>3656.2</v>
-      </c>
-      <c r="J2" t="n">
-        <v>3.34</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
-        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:AIIL","AIIL")</f>
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:GPIL","GPIL")</f>
         <v/>
       </c>
       <c r="B3" t="n">
-        <v>662179</v>
+        <v>8683243</v>
       </c>
       <c r="C3" t="n">
-        <v>131504.6551724138</v>
+        <v>1213165.620689655</v>
       </c>
       <c r="D3" t="n">
-        <v>5.04</v>
-      </c>
-      <c r="E3" t="n">
-        <v>70.69</v>
-      </c>
-      <c r="F3" t="n">
-        <v>936735</v>
-      </c>
-      <c r="G3" t="n">
-        <v>321413.1034482759</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="I3" t="n">
-        <v>507.85</v>
-      </c>
-      <c r="J3" t="n">
-        <v>2.24</v>
+        <v>7.16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:ENRIN","ENRIN")</f>
+        <v/>
+      </c>
+      <c r="B4" t="n">
+        <v>1467156</v>
+      </c>
+      <c r="C4" t="n">
+        <v>228204</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6.43</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:ZYDUSLIFE","ZYDUSLIFE")</f>
+        <v/>
+      </c>
+      <c r="B5" t="n">
+        <v>2612328</v>
+      </c>
+      <c r="C5" t="n">
+        <v>430420.5517241379</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6.07</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:ANTHEM","ANTHEM")</f>
+        <v/>
+      </c>
+      <c r="B6" t="n">
+        <v>1008949</v>
+      </c>
+      <c r="C6" t="n">
+        <v>168324.9655172414</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:PIIND","PIIND")</f>
+        <v/>
+      </c>
+      <c r="B7" t="n">
+        <v>730475</v>
+      </c>
+      <c r="C7" t="n">
+        <v>127434.8965517241</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.73</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:BLS","BLS")</f>
+        <v/>
+      </c>
+      <c r="B8" t="n">
+        <v>2329786</v>
+      </c>
+      <c r="C8" t="n">
+        <v>447989.8620689655</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:ERIS","ERIS")</f>
+        <v/>
+      </c>
+      <c r="B9" t="n">
+        <v>357724</v>
+      </c>
+      <c r="C9" t="n">
+        <v>68958.89655172414</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5.19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:AIIL","AIIL")</f>
+        <v/>
+      </c>
+      <c r="B10" t="n">
+        <v>662179</v>
+      </c>
+      <c r="C10" t="n">
+        <v>131504.6551724138</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:MAPMYINDIA","MAPMYINDIA")</f>
+        <v/>
+      </c>
+      <c r="B11" t="n">
+        <v>316691</v>
+      </c>
+      <c r="C11" t="n">
+        <v>72533.6551724138</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.37</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:CGCL","CGCL")</f>
+        <v/>
+      </c>
+      <c r="B12" t="n">
+        <v>3999407</v>
+      </c>
+      <c r="C12" t="n">
+        <v>914938.3793103448</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4.37</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:GMRAIRPORT","GMRAIRPORT")</f>
+        <v/>
+      </c>
+      <c r="B13" t="n">
+        <v>28214134</v>
+      </c>
+      <c r="C13" t="n">
+        <v>7008074.551724138</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4.03</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:MANKIND","MANKIND")</f>
+        <v/>
+      </c>
+      <c r="B14" t="n">
+        <v>1061305</v>
+      </c>
+      <c r="C14" t="n">
+        <v>269747.8620689655</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.93</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:DIVISLAB","DIVISLAB")</f>
+        <v/>
+      </c>
+      <c r="B15" t="n">
+        <v>605095</v>
+      </c>
+      <c r="C15" t="n">
+        <v>161100</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
         <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:HONAUT","HONAUT")</f>
         <v/>
       </c>
-      <c r="B4" t="n">
+      <c r="B16" t="n">
         <v>8597</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C16" t="n">
         <v>2761.620689655173</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D16" t="n">
         <v>3.11</v>
       </c>
-      <c r="E4" t="n">
-        <v>55.22</v>
-      </c>
-      <c r="F4" t="n">
-        <v>15569</v>
-      </c>
-      <c r="G4" t="n">
-        <v>5665.517241379311</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="I4" t="n">
-        <v>30180</v>
-      </c>
-      <c r="J4" t="n">
-        <v>3.8</v>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <f>HYPERLINK("https://www.tradingview.com/chart/?symbol=NSE:ABCAPITAL","ABCAPITAL")</f>
+        <v/>
+      </c>
+      <c r="B17" t="n">
+        <v>6235154</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2053500.413793104</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.04</v>
       </c>
     </row>
   </sheetData>

</xml_diff>